<commit_message>
By Month tab: add prior/new gross and effective rent dollars
Alongside each trade-out %, show the underlying average rents: prior vs
new gross $ and prior vs new effective $, for both renewals (by
expiration month) and new leases (by re-lease month). TOTAL/AVG row
averages across all leases.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018rGr332ugXyjoVR6V3pSQF
</commit_message>
<xml_diff>
--- a/SeasonsMeridian/analysis/first-turn/Seasons at Meridian - First Turn Analysis.xlsx
+++ b/SeasonsMeridian/analysis/first-turn/Seasons at Meridian - First Turn Analysis.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3978" uniqueCount="1281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3986" uniqueCount="1290">
   <si>
     <t xml:space="preserve">Seasons at Meridian — First Turn of the Rent Roll</t>
   </si>
@@ -3791,13 +3791,40 @@
     <t xml:space="preserve">Month</t>
   </si>
   <si>
+    <t xml:space="preserve">Renewal: Prior Gross $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renewal: New Gross $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renewal: Prior Eff $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renewal: New Eff $</t>
+  </si>
+  <si>
     <t xml:space="preserve">Units Re-Leased (n)</t>
   </si>
   <si>
+    <t xml:space="preserve">New Lease: Prior Gross $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New Lease: New Gross $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New Lease: Prior Eff $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New Lease: New Eff $</t>
+  </si>
+  <si>
     <t xml:space="preserve">Coming Due (not yet expired)</t>
   </si>
   <si>
-    <t xml:space="preserve">Columns B–H are keyed to each initial lease's ORIGINAL first-expiration month (the renewal decision). Columns I–K are keyed to the month the replacement tenant moved in, so re-leases after early lease-breaks appear when they actually happened — not at the broken lease's future expiration date. Column L counts initial leases whose first expiration is still ahead.</t>
+    <t xml:space="preserve">TOTAL / AVG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Columns B–L are keyed to each initial lease's ORIGINAL first-expiration month (the renewal decision). Columns M–S are keyed to the month the replacement tenant moved in, so re-leases after early lease-breaks appear when they actually happened — not at the broken lease's future expiration date. Column T counts initial leases whose first expiration is still ahead. $ columns are simple averages of the leases in that month, so the % columns (avg of per-lease trade-outs) won't exactly equal the ratio of the $ averages. Prior-lease $ for new leases = the departed initial tenant's rent on the same unit. TOTAL/AVG row: counts are sums; $ and % are averages across all leases.</t>
   </si>
   <si>
     <t xml:space="preserve">Seasons at Meridian — First Turn Analysis: Methodology &amp; Caveats</t>
@@ -39105,19 +39132,26 @@
     <tabColor rgb="FF4472C4"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:T31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
         <v>1253</v>
       </c>
@@ -39137,22 +39171,46 @@
         <v>1246</v>
       </c>
       <c r="G1" s="19" t="s">
+        <v>1254</v>
+      </c>
+      <c r="H1" s="19" t="s">
+        <v>1255</v>
+      </c>
+      <c r="I1" s="19" t="s">
         <v>1248</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="J1" s="19" t="s">
+        <v>1256</v>
+      </c>
+      <c r="K1" s="19" t="s">
+        <v>1257</v>
+      </c>
+      <c r="L1" s="19" t="s">
         <v>1249</v>
       </c>
-      <c r="I1" s="19" t="s">
-        <v>1254</v>
-      </c>
-      <c r="J1" s="19" t="s">
+      <c r="M1" s="19" t="s">
+        <v>1258</v>
+      </c>
+      <c r="N1" s="19" t="s">
+        <v>1259</v>
+      </c>
+      <c r="O1" s="19" t="s">
+        <v>1260</v>
+      </c>
+      <c r="P1" s="19" t="s">
         <v>1250</v>
       </c>
-      <c r="K1" s="19" t="s">
+      <c r="Q1" s="19" t="s">
+        <v>1261</v>
+      </c>
+      <c r="R1" s="19" t="s">
+        <v>1262</v>
+      </c>
+      <c r="S1" s="19" t="s">
         <v>1251</v>
       </c>
-      <c r="L1" s="19" t="s">
-        <v>1255</v>
+      <c r="T1" s="19" t="s">
+        <v>1263</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39179,27 +39237,59 @@
         <f aca="false">IF(B2=0,"",C2/B2)</f>
         <v/>
       </c>
-      <c r="G2" s="22" t="str">
+      <c r="G2" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H2" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I2" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H2" s="22" t="str">
+      <c r="J2" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K2" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L2" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="M2" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>1</v>
       </c>
-      <c r="J2" s="22" t="n">
+      <c r="N2" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1475</v>
+      </c>
+      <c r="O2" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1475</v>
+      </c>
+      <c r="P2" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0</v>
       </c>
-      <c r="K2" s="22" t="n">
+      <c r="Q2" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1342</v>
+      </c>
+      <c r="R2" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1290.66666666667</v>
+      </c>
+      <c r="S2" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>-0.0382513661202185</v>
       </c>
-      <c r="L2" s="5" t="n">
+      <c r="T2" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2025-07",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>0</v>
       </c>
@@ -39228,27 +39318,59 @@
         <f aca="false">IF(B3=0,"",C3/B3)</f>
         <v>1</v>
       </c>
-      <c r="G3" s="22" t="n">
+      <c r="G3" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1395</v>
+      </c>
+      <c r="H3" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1415</v>
+      </c>
+      <c r="I3" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0143369175627239</v>
       </c>
-      <c r="H3" s="22" t="n">
+      <c r="J3" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1395</v>
+      </c>
+      <c r="K3" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1415</v>
+      </c>
+      <c r="L3" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0143369175627239</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="M3" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J3" s="22" t="str">
+      <c r="N3" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O3" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P3" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K3" s="22" t="str">
+      <c r="Q3" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R3" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S3" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L3" s="5" t="n">
+      <c r="T3" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2025-08",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>0</v>
       </c>
@@ -39277,27 +39399,59 @@
         <f aca="false">IF(B4=0,"",C4/B4)</f>
         <v>1</v>
       </c>
-      <c r="G4" s="22" t="n">
+      <c r="G4" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1690</v>
+      </c>
+      <c r="H4" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1702.5</v>
+      </c>
+      <c r="I4" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.00902527075812276</v>
       </c>
-      <c r="H4" s="22" t="n">
+      <c r="J4" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1518.5</v>
+      </c>
+      <c r="K4" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1702.5</v>
+      </c>
+      <c r="L4" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.113545359209384</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="M4" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J4" s="22" t="str">
+      <c r="N4" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O4" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P4" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K4" s="22" t="str">
+      <c r="Q4" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R4" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S4" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="T4" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2025-10",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>0</v>
       </c>
@@ -39326,27 +39480,59 @@
         <f aca="false">IF(B5=0,"",C5/B5)</f>
         <v>1</v>
       </c>
-      <c r="G5" s="22" t="n">
+      <c r="G5" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1663.25</v>
+      </c>
+      <c r="H5" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1653</v>
+      </c>
+      <c r="I5" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>-0.00762617409992791</v>
       </c>
-      <c r="H5" s="22" t="n">
+      <c r="J5" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1407.25</v>
+      </c>
+      <c r="K5" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1645.1875</v>
+      </c>
+      <c r="L5" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.167089539712455</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="M5" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J5" s="22" t="str">
+      <c r="N5" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O5" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P5" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K5" s="22" t="str">
+      <c r="Q5" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R5" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S5" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L5" s="5" t="n">
+      <c r="T5" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2025-11",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>0</v>
       </c>
@@ -39375,27 +39561,59 @@
         <f aca="false">IF(B6=0,"",C6/B6)</f>
         <v>0.833333333333333</v>
       </c>
-      <c r="G6" s="22" t="n">
+      <c r="G6" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1860.6</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1871.2</v>
+      </c>
+      <c r="I6" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.00646547731525224</v>
       </c>
-      <c r="H6" s="22" t="n">
+      <c r="J6" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1717</v>
+      </c>
+      <c r="K6" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1871.2</v>
+      </c>
+      <c r="L6" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0923495837207306</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="M6" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J6" s="22" t="str">
+      <c r="N6" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O6" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P6" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K6" s="22" t="str">
+      <c r="Q6" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R6" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S6" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L6" s="5" t="n">
+      <c r="T6" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2025-12",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>0</v>
       </c>
@@ -39424,27 +39642,59 @@
         <f aca="false">IF(B7=0,"",C7/B7)</f>
         <v>0.4</v>
       </c>
-      <c r="G7" s="22" t="n">
+      <c r="G7" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1402.5</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1402.5</v>
+      </c>
+      <c r="I7" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0</v>
       </c>
-      <c r="H7" s="22" t="n">
+      <c r="J7" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1275</v>
+      </c>
+      <c r="K7" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1402.5</v>
+      </c>
+      <c r="L7" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.104517238846551</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="M7" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J7" s="22" t="str">
+      <c r="N7" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O7" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P7" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K7" s="22" t="str">
+      <c r="Q7" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R7" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S7" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L7" s="5" t="n">
+      <c r="T7" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2026-01",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>0</v>
       </c>
@@ -39473,27 +39723,59 @@
         <f aca="false">IF(B8=0,"",C8/B8)</f>
         <v>0.307692307692308</v>
       </c>
-      <c r="G8" s="22" t="n">
+      <c r="G8" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1696.25</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1738.75</v>
+      </c>
+      <c r="I8" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.023464465433921</v>
       </c>
-      <c r="H8" s="22" t="n">
+      <c r="J8" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1647.25</v>
+      </c>
+      <c r="K8" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1738.75</v>
+      </c>
+      <c r="L8" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0540514199658996</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="M8" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>4</v>
       </c>
-      <c r="J8" s="22" t="n">
+      <c r="N8" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1567.25</v>
+      </c>
+      <c r="O8" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1583.25</v>
+      </c>
+      <c r="P8" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0103972266871042</v>
       </c>
-      <c r="K8" s="22" t="n">
+      <c r="Q8" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1456.5</v>
+      </c>
+      <c r="R8" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1583.25</v>
+      </c>
+      <c r="S8" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0868153210708264</v>
       </c>
-      <c r="L8" s="5" t="n">
+      <c r="T8" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2026-02",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>0</v>
       </c>
@@ -39522,27 +39804,59 @@
         <f aca="false">IF(B9=0,"",C9/B9)</f>
         <v>0.294117647058824</v>
       </c>
-      <c r="G9" s="22" t="n">
+      <c r="G9" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1717</v>
+      </c>
+      <c r="H9" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1717</v>
+      </c>
+      <c r="I9" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0</v>
       </c>
-      <c r="H9" s="22" t="n">
+      <c r="J9" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1642.2</v>
+      </c>
+      <c r="K9" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1717</v>
+      </c>
+      <c r="L9" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0505093280644094</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="M9" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>18</v>
       </c>
-      <c r="J9" s="22" t="n">
+      <c r="N9" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1616.94444444444</v>
+      </c>
+      <c r="O9" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1657.61111111111</v>
+      </c>
+      <c r="P9" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0310783863268381</v>
       </c>
-      <c r="K9" s="22" t="n">
+      <c r="Q9" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1530.38888888889</v>
+      </c>
+      <c r="R9" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1638.03086419753</v>
+      </c>
+      <c r="S9" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0891817750221162</v>
       </c>
-      <c r="L9" s="5" t="n">
+      <c r="T9" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2026-03",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>0</v>
       </c>
@@ -39571,27 +39885,59 @@
         <f aca="false">IF(B10=0,"",C10/B10)</f>
         <v>0.555555555555556</v>
       </c>
-      <c r="G10" s="22" t="n">
+      <c r="G10" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1827.4</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1864.4</v>
+      </c>
+      <c r="I10" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0204949768511321</v>
       </c>
-      <c r="H10" s="22" t="n">
+      <c r="J10" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1745.2</v>
+      </c>
+      <c r="K10" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1864.4</v>
+      </c>
+      <c r="L10" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.071950531639504</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="M10" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>11</v>
       </c>
-      <c r="J10" s="22" t="n">
+      <c r="N10" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1770.45454545455</v>
+      </c>
+      <c r="O10" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1839.90909090909</v>
+      </c>
+      <c r="P10" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0376187388849813</v>
       </c>
-      <c r="K10" s="22" t="n">
+      <c r="Q10" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1637.54545454545</v>
+      </c>
+      <c r="R10" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1759.2446969697</v>
+      </c>
+      <c r="S10" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0749579853350263</v>
       </c>
-      <c r="L10" s="5" t="n">
+      <c r="T10" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2026-04",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>0</v>
       </c>
@@ -39620,27 +39966,59 @@
         <f aca="false">IF(B11=0,"",C11/B11)</f>
         <v>0.428571428571429</v>
       </c>
-      <c r="G11" s="22" t="n">
+      <c r="G11" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1695.55555555556</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1731.66666666667</v>
+      </c>
+      <c r="I11" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0225948035426665</v>
       </c>
-      <c r="H11" s="22" t="n">
+      <c r="J11" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1531.80876068376</v>
+      </c>
+      <c r="K11" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1723.14102564103</v>
+      </c>
+      <c r="L11" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.129040796316841</v>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="M11" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>9</v>
       </c>
-      <c r="J11" s="22" t="n">
+      <c r="N11" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1806.88888888889</v>
+      </c>
+      <c r="O11" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1844.77777777778</v>
+      </c>
+      <c r="P11" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0251790419719461</v>
       </c>
-      <c r="K11" s="22" t="n">
+      <c r="Q11" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1687.33333333333</v>
+      </c>
+      <c r="R11" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1811.39814814815</v>
+      </c>
+      <c r="S11" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0863822183308243</v>
       </c>
-      <c r="L11" s="5" t="n">
+      <c r="T11" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2026-05",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>0</v>
       </c>
@@ -39669,27 +40047,59 @@
         <f aca="false">IF(B12=0,"",C12/B12)</f>
         <v>0.5</v>
       </c>
-      <c r="G12" s="22" t="n">
+      <c r="G12" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1761</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1792.78571428571</v>
+      </c>
+      <c r="I12" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0181714490797891</v>
       </c>
-      <c r="H12" s="22" t="n">
+      <c r="J12" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1635.8231292517</v>
+      </c>
+      <c r="K12" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1792.78571428571</v>
+      </c>
+      <c r="L12" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0973498573750208</v>
       </c>
-      <c r="I12" s="5" t="n">
+      <c r="M12" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>16</v>
       </c>
-      <c r="J12" s="22" t="n">
+      <c r="N12" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1875.25</v>
+      </c>
+      <c r="O12" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1956.9375</v>
+      </c>
+      <c r="P12" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0485754774470234</v>
       </c>
-      <c r="K12" s="22" t="n">
+      <c r="Q12" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1732.25</v>
+      </c>
+      <c r="R12" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1897.93273809524</v>
+      </c>
+      <c r="S12" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.102370045388463</v>
       </c>
-      <c r="L12" s="5" t="n">
+      <c r="T12" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2026-06",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>0</v>
       </c>
@@ -39718,27 +40128,59 @@
         <f aca="false">IF(B13=0,"",C13/B13)</f>
         <v>0.216216216216216</v>
       </c>
-      <c r="G13" s="22" t="n">
+      <c r="G13" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1718.25</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1755.5</v>
+      </c>
+      <c r="I13" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.0240672301167577</v>
       </c>
-      <c r="H13" s="22" t="n">
+      <c r="J13" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1594.16666666667</v>
+      </c>
+      <c r="K13" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1755.5</v>
+      </c>
+      <c r="L13" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.100840297066339</v>
       </c>
-      <c r="I13" s="5" t="n">
+      <c r="M13" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>30</v>
       </c>
-      <c r="J13" s="22" t="n">
+      <c r="N13" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1755.23333333333</v>
+      </c>
+      <c r="O13" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1889.8</v>
+      </c>
+      <c r="P13" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.079155111880287</v>
       </c>
-      <c r="K13" s="22" t="n">
+      <c r="Q13" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1645.965</v>
+      </c>
+      <c r="R13" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1873.30747126437</v>
+      </c>
+      <c r="S13" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.146001009020784</v>
       </c>
-      <c r="L13" s="5" t="n">
+      <c r="T13" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2026-07",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>0</v>
       </c>
@@ -39767,27 +40209,59 @@
         <f aca="false">IF(B14=0,"",C14/B14)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="22" t="str">
+      <c r="G14" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H14" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H14" s="22" t="str">
+      <c r="J14" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="M14" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>3</v>
       </c>
-      <c r="J14" s="22" t="n">
+      <c r="N14" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1955.33333333333</v>
+      </c>
+      <c r="O14" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>2205.66666666667</v>
+      </c>
+      <c r="P14" s="22" t="n">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v>0.122496731861349</v>
       </c>
-      <c r="K14" s="22" t="str">
+      <c r="Q14" s="16" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1808.59444444444</v>
+      </c>
+      <c r="R14" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S14" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L14" s="5" t="n">
+      <c r="T14" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2026-08",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>30</v>
       </c>
@@ -39816,27 +40290,59 @@
         <f aca="false">IF(B15=0,"",C15/B15)</f>
         <v/>
       </c>
-      <c r="G15" s="22" t="str">
+      <c r="G15" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H15" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H15" s="22" t="str">
+      <c r="J15" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K15" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="M15" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J15" s="22" t="str">
+      <c r="N15" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O15" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P15" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K15" s="22" t="str">
+      <c r="Q15" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R15" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S15" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L15" s="5" t="n">
+      <c r="T15" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2026-09",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>14</v>
       </c>
@@ -39865,27 +40371,59 @@
         <f aca="false">IF(B16=0,"",C16/B16)</f>
         <v/>
       </c>
-      <c r="G16" s="22" t="str">
+      <c r="G16" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H16" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H16" s="22" t="str">
+      <c r="J16" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="M16" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J16" s="22" t="str">
+      <c r="N16" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O16" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P16" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K16" s="22" t="str">
+      <c r="Q16" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R16" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S16" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L16" s="5" t="n">
+      <c r="T16" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2026-10",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>20</v>
       </c>
@@ -39914,27 +40452,59 @@
         <f aca="false">IF(B17=0,"",C17/B17)</f>
         <v/>
       </c>
-      <c r="G17" s="22" t="str">
+      <c r="G17" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H17" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I17" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H17" s="22" t="str">
+      <c r="J17" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="M17" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J17" s="22" t="str">
+      <c r="N17" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O17" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P17" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K17" s="22" t="str">
+      <c r="Q17" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R17" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S17" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L17" s="5" t="n">
+      <c r="T17" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2026-11",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>15</v>
       </c>
@@ -39963,27 +40533,59 @@
         <f aca="false">IF(B18=0,"",C18/B18)</f>
         <v/>
       </c>
-      <c r="G18" s="22" t="str">
+      <c r="G18" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H18" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I18" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H18" s="22" t="str">
+      <c r="J18" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K18" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="M18" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J18" s="22" t="str">
+      <c r="N18" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O18" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P18" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K18" s="22" t="str">
+      <c r="Q18" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R18" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S18" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L18" s="5" t="n">
+      <c r="T18" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2026-12",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>12</v>
       </c>
@@ -40012,27 +40614,59 @@
         <f aca="false">IF(B19=0,"",C19/B19)</f>
         <v/>
       </c>
-      <c r="G19" s="22" t="str">
+      <c r="G19" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H19" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I19" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H19" s="22" t="str">
+      <c r="J19" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="M19" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J19" s="22" t="str">
+      <c r="N19" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O19" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P19" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K19" s="22" t="str">
+      <c r="Q19" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R19" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S19" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L19" s="5" t="n">
+      <c r="T19" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2027-01",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>6</v>
       </c>
@@ -40061,27 +40695,59 @@
         <f aca="false">IF(B20=0,"",C20/B20)</f>
         <v/>
       </c>
-      <c r="G20" s="22" t="str">
+      <c r="G20" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H20" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I20" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H20" s="22" t="str">
+      <c r="J20" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K20" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I20" s="5" t="n">
+      <c r="M20" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J20" s="22" t="str">
+      <c r="N20" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O20" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P20" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K20" s="22" t="str">
+      <c r="Q20" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R20" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S20" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L20" s="5" t="n">
+      <c r="T20" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2027-02",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>11</v>
       </c>
@@ -40110,27 +40776,59 @@
         <f aca="false">IF(B21=0,"",C21/B21)</f>
         <v/>
       </c>
-      <c r="G21" s="22" t="str">
+      <c r="G21" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H21" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I21" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H21" s="22" t="str">
+      <c r="J21" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K21" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I21" s="5" t="n">
+      <c r="M21" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J21" s="22" t="str">
+      <c r="N21" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O21" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P21" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K21" s="22" t="str">
+      <c r="Q21" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R21" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S21" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L21" s="5" t="n">
+      <c r="T21" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2027-03",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>12</v>
       </c>
@@ -40159,27 +40857,59 @@
         <f aca="false">IF(B22=0,"",C22/B22)</f>
         <v/>
       </c>
-      <c r="G22" s="22" t="str">
+      <c r="G22" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H22" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I22" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H22" s="22" t="str">
+      <c r="J22" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K22" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L22" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I22" s="5" t="n">
+      <c r="M22" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J22" s="22" t="str">
+      <c r="N22" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O22" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P22" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K22" s="22" t="str">
+      <c r="Q22" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R22" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S22" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L22" s="5" t="n">
+      <c r="T22" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2027-04",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>7</v>
       </c>
@@ -40208,27 +40938,59 @@
         <f aca="false">IF(B23=0,"",C23/B23)</f>
         <v/>
       </c>
-      <c r="G23" s="22" t="str">
+      <c r="G23" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H23" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I23" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H23" s="22" t="str">
+      <c r="J23" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K23" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I23" s="5" t="n">
+      <c r="M23" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J23" s="22" t="str">
+      <c r="N23" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O23" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P23" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K23" s="22" t="str">
+      <c r="Q23" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R23" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S23" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L23" s="5" t="n">
+      <c r="T23" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2027-05",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>6</v>
       </c>
@@ -40257,27 +41019,59 @@
         <f aca="false">IF(B24=0,"",C24/B24)</f>
         <v/>
       </c>
-      <c r="G24" s="22" t="str">
+      <c r="G24" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H24" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I24" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H24" s="22" t="str">
+      <c r="J24" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K24" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I24" s="5" t="n">
+      <c r="M24" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J24" s="22" t="str">
+      <c r="N24" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O24" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P24" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K24" s="22" t="str">
+      <c r="Q24" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R24" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S24" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L24" s="5" t="n">
+      <c r="T24" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2027-06",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>4</v>
       </c>
@@ -40306,34 +41100,66 @@
         <f aca="false">IF(B25=0,"",C25/B25)</f>
         <v/>
       </c>
-      <c r="G25" s="22" t="str">
+      <c r="G25" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$J$2:$J$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="H25" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$J$2:$J$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="I25" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$J$2:$J$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="H25" s="22" t="str">
+      <c r="J25" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$J$2:$J$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="K25" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$J$2:$J$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="L25" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$J$2:$J$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="I25" s="5" t="n">
+      <c r="M25" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$AP$2:$AP$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out")</f>
         <v>0</v>
       </c>
-      <c r="J25" s="22" t="str">
+      <c r="N25" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$AP$2:$AP$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="O25" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$AP$2:$AP$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="P25" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$AP$2:$AP$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="K25" s="22" t="str">
+      <c r="Q25" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$AP$2:$AP$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="R25" s="16" t="str">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$AP$2:$AP$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v/>
+      </c>
+      <c r="S25" s="22" t="str">
         <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$AP$2:$AP$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
         <v/>
       </c>
-      <c r="L25" s="5" t="n">
+      <c r="T25" s="5" t="n">
         <f aca="false">COUNTIFS('Unit Ledger'!$J$2:$J$315,"2027-07",'Unit Ledger'!$Q$2:$Q$315,"Not Yet Expired")</f>
         <v>2</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>1252</v>
+        <v>1264</v>
       </c>
       <c r="B26" s="7" t="n">
         <f aca="false">SUM(B2:B25)</f>
@@ -40355,18 +41181,66 @@
         <f aca="false">IF(B26=0,"",C26/B26)</f>
         <v>0.415584415584416</v>
       </c>
-      <c r="I26" s="7" t="n">
-        <f aca="false">SUM(I2:I25)</f>
+      <c r="G26" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1731.875</v>
+      </c>
+      <c r="H26" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$Y$2:$Y$315,'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1757.890625</v>
+      </c>
+      <c r="I26" s="13" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AC$2:$AC$315,'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>0.015364205303713</v>
+      </c>
+      <c r="J26" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1607.6427498283</v>
+      </c>
+      <c r="K26" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AA$2:$AA$315,'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1756.20342548077</v>
+      </c>
+      <c r="L26" s="13" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AD$2:$AD$315,'Unit Ledger'!$Q$2:$Q$315,"Renewed",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>0.0953095839740832</v>
+      </c>
+      <c r="M26" s="7" t="n">
+        <f aca="false">SUM(M2:M25)</f>
         <v>92</v>
       </c>
-      <c r="L26" s="7" t="n">
-        <f aca="false">SUM(L2:L25)</f>
+      <c r="N26" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$L$2:$L$315,'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1747.82692307692</v>
+      </c>
+      <c r="O26" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AJ$2:$AJ$315,'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1838.14130434783</v>
+      </c>
+      <c r="P26" s="13" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AM$2:$AM$315,'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>0.0517474843180309</v>
+      </c>
+      <c r="Q26" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$N$2:$N$315,'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1634.37844551282</v>
+      </c>
+      <c r="R26" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AL$2:$AL$315,'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>1789.26520111833</v>
+      </c>
+      <c r="S26" s="13" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS('Unit Ledger'!$AN$2:$AN$315,'Unit Ledger'!$Q$2:$Q$315,"Moved Out",'Unit Ledger'!$V$2:$V$315,"&lt;&gt;Y"),"")</f>
+        <v>0.106684200682296</v>
+      </c>
+      <c r="T26" s="7" t="n">
+        <f aca="false">SUM(T2:T25)</f>
         <v>139</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="30" t="s">
-        <v>1256</v>
+        <v>1265</v>
       </c>
       <c r="B28" s="30"/>
       <c r="C28" s="30"/>
@@ -40379,6 +41253,14 @@
       <c r="J28" s="30"/>
       <c r="K28" s="30"/>
       <c r="L28" s="30"/>
+      <c r="M28" s="30"/>
+      <c r="N28" s="30"/>
+      <c r="O28" s="30"/>
+      <c r="P28" s="30"/>
+      <c r="Q28" s="30"/>
+      <c r="R28" s="30"/>
+      <c r="S28" s="30"/>
+      <c r="T28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30"/>
@@ -40393,6 +41275,14 @@
       <c r="J29" s="30"/>
       <c r="K29" s="30"/>
       <c r="L29" s="30"/>
+      <c r="M29" s="30"/>
+      <c r="N29" s="30"/>
+      <c r="O29" s="30"/>
+      <c r="P29" s="30"/>
+      <c r="Q29" s="30"/>
+      <c r="R29" s="30"/>
+      <c r="S29" s="30"/>
+      <c r="T29" s="30"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="30"/>
@@ -40407,10 +41297,40 @@
       <c r="J30" s="30"/>
       <c r="K30" s="30"/>
       <c r="L30" s="30"/>
+      <c r="M30" s="30"/>
+      <c r="N30" s="30"/>
+      <c r="O30" s="30"/>
+      <c r="P30" s="30"/>
+      <c r="Q30" s="30"/>
+      <c r="R30" s="30"/>
+      <c r="S30" s="30"/>
+      <c r="T30" s="30"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="30"/>
+      <c r="B31" s="30"/>
+      <c r="C31" s="30"/>
+      <c r="D31" s="30"/>
+      <c r="E31" s="30"/>
+      <c r="F31" s="30"/>
+      <c r="G31" s="30"/>
+      <c r="H31" s="30"/>
+      <c r="I31" s="30"/>
+      <c r="J31" s="30"/>
+      <c r="K31" s="30"/>
+      <c r="L31" s="30"/>
+      <c r="M31" s="30"/>
+      <c r="N31" s="30"/>
+      <c r="O31" s="30"/>
+      <c r="P31" s="30"/>
+      <c r="Q31" s="30"/>
+      <c r="R31" s="30"/>
+      <c r="S31" s="30"/>
+      <c r="T31" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A28:L30"/>
+    <mergeCell ref="A28:T31"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -40436,7 +41356,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="31" t="s">
-        <v>1257</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40444,27 +41364,27 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="33" t="s">
-        <v>1258</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="32" t="s">
-        <v>1259</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>1260</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>1261</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>1262</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40472,22 +41392,22 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="33" t="s">
-        <v>1263</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>1264</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>1265</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>1266</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40495,27 +41415,27 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="33" t="s">
-        <v>1267</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>1268</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>1269</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>1270</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>1271</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40523,27 +41443,27 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="33" t="s">
-        <v>1272</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>1273</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>1274</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>1275</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>1276</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40551,22 +41471,22 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="33" t="s">
-        <v>1277</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>1278</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>1279</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>1280</v>
+        <v>1289</v>
       </c>
     </row>
   </sheetData>

</xml_diff>